<commit_message>
Added log , extent report and screenshot utility and integrated in class
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/AllDetails.xlsx
+++ b/src/test/resources/testData/AllDetails.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2464425_cognizant_com/Documents/Desktop/AUTOMATION/JAVA/PROJECT/MajorProject-Automation/src/test/resources/testData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="11_1C2DCCB743D214D3C6AA5E811A286F0A5940F7A3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E913D97-401B-41B9-BC4C-15D61C3DA661}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="11_1C2DCCB743D214D3C6AA5E811A286F0A5940F7A3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73DFB69C-2F8D-4238-BDB7-62BE993F2C91}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AppointmentFormValidData" sheetId="1" r:id="rId1"/>
     <sheet name="AppointmentFormInvalidData" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -109,10 +110,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -490,4 +487,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06BE5F1C-84F5-4E44-8C3D-88DCB3741296}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added excel file, screenshot and logs
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/AllDetails.xlsx
+++ b/src/test/resources/testData/AllDetails.xlsx
@@ -5,23 +5,25 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2464425_cognizant_com/Documents/Desktop/AUTOMATION/JAVA/PROJECT/MajorProject-Automation/src/test/resources/testData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2464529_cognizant_com/Documents/Desktop/practo_project/practo-web-automation/src/test/resources/testData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="11_1C2DCCB743D214D3C6AA5E811A286F0A5940F7A3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E913D97-401B-41B9-BC4C-15D61C3DA661}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="11_1C2DCCB743D214D3C6AA5E811A286F0A5940F7A3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8FF6D2B-7E68-445C-A30F-288E80147639}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AppointmentFormValidData" sheetId="1" r:id="rId1"/>
     <sheet name="AppointmentFormInvalidData" sheetId="2" r:id="rId2"/>
+    <sheet name="DemoFormInvalidData" sheetId="3" r:id="rId3"/>
+    <sheet name="DemoFormValidData" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="11">
   <si>
     <t>Name</t>
   </si>
@@ -33,13 +35,34 @@
   </si>
   <si>
     <t>13213bakdfbdka</t>
+  </si>
+  <si>
+    <t>OrganizationName</t>
+  </si>
+  <si>
+    <t>EmailId</t>
+  </si>
+  <si>
+    <t>Samidha</t>
+  </si>
+  <si>
+    <t>cts</t>
+  </si>
+  <si>
+    <t>Cognizant</t>
+  </si>
+  <si>
+    <t>abc@xyz</t>
+  </si>
+  <si>
+    <t>samidha@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -52,6 +75,14 @@
       <color indexed="8"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -86,16 +117,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -490,4 +524,102 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83267885-82C2-4EAD-B1CB-1C15ACCABC99}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="27.54296875" customWidth="1"/>
+    <col min="2" max="2" width="39.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>987655</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" xr:uid="{63E40D88-678A-48F4-97B8-39F623B55B30}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5FDF007-C92B-480C-B134-45EC911F9E68}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.7265625" customWidth="1"/>
+    <col min="2" max="2" width="37.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>9898989898</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" xr:uid="{75E5F89A-5955-46C6-BCC0-ED1E6D0E1ACA}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
UPDATE EXCEL AND FIXED TESTCASES
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/AllDetails.xlsx
+++ b/src/test/resources/testData/AllDetails.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2464425_cognizant_com/Documents/Desktop/AUTOMATION/JAVA/PROJECT/MajorProject-Automation/src/test/resources/testData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="11_1C2DCCB743D214D3C6AA5E811A286F0A5940F7A3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73DFB69C-2F8D-4238-BDB7-62BE993F2C91}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="11_1C2DCCB743D214D3C6AA5E811A286F0A5940F7A3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C383CA38-A832-49CD-AD5E-F1DD1C88B32C}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AppointmentFormValidData" sheetId="1" r:id="rId1"/>
     <sheet name="AppointmentFormInvalidData" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
+    <sheet name="DemoFormInvalidData" sheetId="4" r:id="rId3"/>
+    <sheet name="DemoFormValidData " sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="12">
   <si>
     <t>Name</t>
   </si>
@@ -34,13 +35,37 @@
   </si>
   <si>
     <t>13213bakdfbdka</t>
+  </si>
+  <si>
+    <t>OrganizationName</t>
+  </si>
+  <si>
+    <t>EmailId</t>
+  </si>
+  <si>
+    <t>sam</t>
+  </si>
+  <si>
+    <t>cts</t>
+  </si>
+  <si>
+    <t>dsa@xyz.com</t>
+  </si>
+  <si>
+    <t>Jhon</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>jhonamazon@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -53,6 +78,14 @@
       <color indexed="8"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -87,16 +120,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -110,6 +146,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -490,10 +530,98 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06BE5F1C-84F5-4E44-8C3D-88DCB3741296}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE8DE462-2339-4272-A58C-725C4AA928AA}">
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="21.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>822828</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" xr:uid="{B9AD54E5-5383-49C0-87B8-D57EEAF0D880}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62ADE2F6-CAEE-46A0-BAD9-857E73BD3DC8}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21.36328125" customWidth="1"/>
+    <col min="2" max="2" width="19.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>8228288768</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" xr:uid="{360C970B-0F34-4A03-A98F-915B49D87183}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added testdata to gitignore
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/AllDetails.xlsx
+++ b/src/test/resources/testData/AllDetails.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2464425_cognizant_com/Documents/Desktop/AUTOMATION/JAVA/PROJECT/MajorProject-Automation/src/test/resources/testData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="11_1C2DCCB743D214D3C6AA5E811A286F0A5940F7A3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC1F63B6-6BA3-4348-BE5F-8EB739441B48}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="11_1C2DCCB743D214D3C6AA5E811A286F0A5940F7A3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05B77743-C0BB-4D76-9D9C-9E852C200741}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="15">
   <si>
     <t>Name</t>
   </si>
@@ -478,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.90625" customWidth="1"/>
@@ -515,6 +515,11 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed DiagnosticPage aflter conflict resolving
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/AllDetails.xlsx
+++ b/src/test/resources/testData/AllDetails.xlsx
@@ -8,21 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2464425_cognizant_com/Documents/Desktop/AUTOMATION/JAVA/PROJECT/MajorProject-Automation/src/test/resources/testData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="11_1C2DCCB743D214D3C6AA5E811A286F0A5940F7A3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73DFB69C-2F8D-4238-BDB7-62BE993F2C91}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="11_1C2DCCB743D214D3C6AA5E811A286F0A5940F7A3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E181207-7437-4E66-BA70-0159B395CECD}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AppointmentFormValidData" sheetId="1" r:id="rId1"/>
     <sheet name="AppointmentFormInvalidData" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
+    <sheet name="DemoFormInvalidData" sheetId="3" r:id="rId3"/>
+    <sheet name="DemoFormValidData" sheetId="5" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="10">
   <si>
     <t>Name</t>
   </si>
@@ -34,13 +36,31 @@
   </si>
   <si>
     <t>13213bakdfbdka</t>
+  </si>
+  <si>
+    <t>OrganizationName</t>
+  </si>
+  <si>
+    <t>EmailId</t>
+  </si>
+  <si>
+    <t>Samidha</t>
+  </si>
+  <si>
+    <t>cts</t>
+  </si>
+  <si>
+    <t>Samidha@xyz</t>
+  </si>
+  <si>
+    <t>Samidha@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -53,6 +73,14 @@
       <color indexed="8"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -87,16 +115,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -491,6 +522,104 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06BE5F1C-84F5-4E44-8C3D-88DCB3741296}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.08984375" customWidth="1"/>
+    <col min="2" max="2" width="14.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>989898</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" xr:uid="{2364CC1C-12EA-4D7D-B402-8344500BD67F}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84644DAF-F0B5-44BF-90D9-8D61A8C2973E}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.08984375" customWidth="1"/>
+    <col min="2" max="2" width="40.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>9898989898</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" xr:uid="{DFAA966F-5F7C-4ADA-A805-F4AFA7EFB7AB}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{909B5B3C-F652-47D7-A507-7A3B07850AC2}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>

</xml_diff>